<commit_message>
ci(dev): publish dev build from dc4d85b66043a9ed85f8c998a6ef9302d60d8994 dc4d85b66043a9ed85f8c998a6ef9302d60d8994
</commit_message>
<xml_diff>
--- a/dev/StructureDefinition-ereferral-provenance.xlsx
+++ b/dev/StructureDefinition-ereferral-provenance.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-17T05:47:03+00:00</t>
+    <t>2026-06-17T10:39:22+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -491,7 +491,7 @@
     <t>The Reference(s) that were generated or updated by the activity described in this resource. A provenance can point to more than one target if multiple resources were created/updated by a single activity.</t>
   </si>
   <si>
-    <t>See the [PH Core Provenance Profile](https://build.fhir.org/ig/jgsuess/ph-core/StructureDefinition-ph-core-provenance.html) for guidance on supported resource types.</t>
+    <t>See the [PH Core Provenance Profile](file:///home/runner/work/ph-core/ph-core/output/StructureDefinition-ph-core-provenance.html) for guidance on supported resource types.</t>
   </si>
   <si>
     <t>./outboundRelationship[isNormalActRelationship() and typeCode=SUBJ]/target  OR  ./participation[isNormalParticipation() and typeCode=SBJ]/role  OR  ./participation[isNormalParticipation() and typeCode=SBJ]/role[isNormalRole()]/player</t>

</xml_diff>